<commit_message>
Filters for exams dates applied, seems working
</commit_message>
<xml_diff>
--- a/templates/entrance_exams_dict.xlsx
+++ b/templates/entrance_exams_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tijuanap\Programs\HSE_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF442397-DAE1-49DD-ABC9-84ED3AD58C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08069AF9-5CF5-45E5-A7E7-CC4DBB54113B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{75D8F8DD-9DF7-456C-8EF8-8325B40ADD81}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{75D8F8DD-9DF7-456C-8EF8-8325B40ADD81}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="88">
   <si>
     <t>Предмет</t>
   </si>
@@ -297,6 +297,12 @@
   </si>
   <si>
     <t>Инженерия данных</t>
+  </si>
+  <si>
+    <t>Портфолио: психологическое консультирование</t>
+  </si>
+  <si>
+    <t>Собеседование: проектирование и разработка высоконагруженных информационных систем</t>
   </si>
 </sst>
 </file>
@@ -367,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -377,6 +383,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -713,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B879D3-9294-417C-8628-265338D2A4C7}">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="92.85546875" bestFit="1" customWidth="1"/>
@@ -952,148 +962,164 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" t="s">
-        <v>53</v>
+    <row r="30" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B35" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+      <c r="A36" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B37" s="3" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>65</v>
-      </c>
-      <c r="B37" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>71</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B43" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B44" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="8" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B46" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B48" s="2" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>